<commit_message>
uploading multiple files at once and adding an excel button so the information transfers over
</commit_message>
<xml_diff>
--- a/data/specs/sample_specs.xlsx
+++ b/data/specs/sample_specs.xlsx
@@ -518,12 +518,12 @@
     <row r="757">
       <c r="A757" t="inlineStr">
         <is>
-          <t>creaseless creamy cnclr-57H rich honey</t>
+          <t>tartelette XL tubing mascara</t>
         </is>
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>OM51</t>
+          <t>CN42</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>FG14816-UN</t>
+          <t>FG13234-UN</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">

</xml_diff>

<commit_message>
reedited files because didn't work before and added gitignore
</commit_message>
<xml_diff>
--- a/data/specs/sample_specs.xlsx
+++ b/data/specs/sample_specs.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>CN42</t>
+          <t>creaseless setting powder-yellow</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
@@ -533,10 +533,15 @@
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>FG13234-UN</t>
+          <t>10/14/2025</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">
+        <is>
+          <t>FG13725-U2</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
         <is>
           <t>3</t>
         </is>

</xml_diff>